<commit_message>
Test Data Excel file updated
</commit_message>
<xml_diff>
--- a/src/test/resources/testData.xlsx
+++ b/src/test/resources/testData.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">harioz</t>
   </si>
   <si>
-    <t xml:space="preserve">test@mail.com</t>
+    <t xml:space="preserve">harioz1515@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">password</t>
@@ -58,6 +58,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -79,6 +80,7 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -123,12 +125,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -259,58 +265,58 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>626189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9025633416</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="test@mail.com"/>
+    <hyperlink ref="A2" r:id="rId1" display="harioz1515@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>